<commit_message>
Fix Template 11 Excel repair prompt — remove invalid empty numeric cells
openpyxl was writing cells with t="n" (numeric type) but no value element,
which triggers Excel's "We found a problem with some content" recovery
dialog. Patched XML to remove the type attribute from 37 empty cells.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_11_Priority_Scoring_Reference.xlsx
+++ b/templates/Template_11_Priority_Scoring_Reference.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,14 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="007A7A7A"/>
+      <i val="1"/>
+      <color rgb="005C5C5C"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -50,12 +45,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001B4965"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -82,32 +78,39 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D4D0C8"/>
+        <color rgb="00D6D6D6"/>
       </left>
       <right style="thin">
-        <color rgb="00D4D0C8"/>
+        <color rgb="00D6D6D6"/>
       </right>
       <top style="thin">
-        <color rgb="00D4D0C8"/>
+        <color rgb="00D6D6D6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D4D0C8"/>
+        <color rgb="00D6D6D6"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,6 +491,9 @@
           <t>PRIORITY SCORING SCALE (0-5)</t>
         </is>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -495,144 +501,153 @@
           <t>Used by the 8-input weighted composite scoring system</t>
         </is>
       </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Don Bosco Prep Courses</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>PROTECTED / MANDATED</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Cannot be bumped. Federal/state mandates, IEP requirements.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>AP 2-D Art and Design (254), AP 3-D Art and Design (255), AP Art History (764), AP Biology (551), AP Business with Personal Finance (729), AP Calc AB (453), AP Calc BC (455), AP Chemistry (553) ... (+55 more)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Required Core / Graduation</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Required for graduation. Must be placed before lower priorities.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Algebra I (410), Algebra I (412), American Literature (120), American Literature (122), British Literature (130), British Literature (132), Catholic Social Teaching (849), Composition &amp; Literature (110) ... (+10 more)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sequence / Honors / AP</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Academic sequence or advanced track. High placement priority.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Algebra I H (411), Algebra II/Trig (430), Algebra II/Trig (432), Algebra II/Trig H (431), American Literature H (121), Anatomy/Physiology (542), Anatomy/Physiology H (543), Biology H (511) ... (+21 more)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Departmental Core</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Core departmental offerings. Important but not graduation-critical.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Biology (510), CPR-AED Training/PE (631), Chemistry (520), Driver's Ed/PE (620), Health/PE (610), Nutrition &amp; Fitness/PE (642), Physics (530), Psychology (741) ... (+5 more)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Standard Elective</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Elective courses. Placed after higher priorities satisfied.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>American Government &amp; Politics (751), Bloomberg Market Concepts (758), Business Concepts (726), Business Law (732), Digital Media (2054), Earth Science (500), Economics (742), Forensics (546) ... (+10 more)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Free Elective / Low Demand</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Nice-to-have. Placed last. Acceptable loss if conflicts exist.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
+      <c r="D10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -662,6 +677,11 @@
           <t>8-INPUT WEIGHTED COMPOSITE SCORING SYSTEM</t>
         </is>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -669,278 +689,299 @@
           <t>Each student-course placement is scored using these 8 inputs</t>
         </is>
       </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Course Flexibility Priority</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>CFP</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>How flexible is this course in scheduling?</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Current Year Required Priority</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CYRP</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Is this course required THIS year?</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Student Special Priority</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>SSP</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Does this student have special scheduling needs?</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Student Profile</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Master Teacher Priority</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>MTP</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Is the assigned teacher highly constrained?</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Teacher Profile</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Course-Teacher Affinity Priority</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>CTAP</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>How strong is the teacher-course match?</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Course + Teacher Profile</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Teacher Lock</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Is the teacher locked to specific periods?</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Teacher Profile</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Period Lock</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Is this course locked to a specific period?</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Room Lock</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>RL</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Is this course locked to a specific room?</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Room Profile</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -948,10 +989,14 @@
           <t>Maximum Weighted Sum:</t>
         </is>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="5">
         <f> 5x(1.0 + 1.5 + 2.0 + 1.0 + 1.5 + 2.0 + 2.0 + 1.5) = 62.5</f>
         <v/>
       </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rebuild Template 11 from scratch with live engine priority data
Regenerated from course_priorities.json and priority_assignments.json
to ensure correct structure. Includes all 6 priority levels with full
course lists and 8-input weight reference with composite formula.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_11_Priority_Scoring_Reference.xlsx
+++ b/templates/Template_11_Priority_Scoring_Reference.xlsx
@@ -40,10 +40,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -51,6 +47,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -102,10 +102,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -480,9 +480,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,9 +491,6 @@
           <t>PRIORITY SCORING SCALE (0-5)</t>
         </is>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -501,155 +498,150 @@
           <t>Used by the 8-input weighted composite scoring system</t>
         </is>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Don Bosco Prep Courses</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>PROTECTED / MANDATED</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Cannot be bumped. Federal/state mandates, IEP requirements.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>AP 2-D Art and Design (254), AP 3-D Art and Design (255), AP Art History (764), AP Biology (551), AP Business with Personal Finance (729), AP Calc AB (453), AP Calc BC (455), AP Chemistry (553) ... (+55 more)</t>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>AP / Singleton / Non-Substitutable</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Highest priority. AP courses, unique singletons, cohort-pinned courses. Cannot be left unscheduled.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>AP Seminar (129), AP English Language (139), Creative Writing (143), AP English Literature (149), Introduction to Guitar (201), Guitar Ensemble (203), Band (206), String Orchestra (209), Music Theory (220), Tech Theater Level 1 (225), Adv Theater Production (228), Studio Art II (242), Studio Art III (243), Adv Drawing (248), Adv Painting (249), AP Drawing (253), AP 2-D Art and Design (254), AP 3-D Art and Design (255), Spanish I H (311), Latin I H (315), Italian II H (323), Latin II H (327), Italian III (332), Latin III H (339), AP Spanish (351), AP Italian (352), AP Latin (359), Adv Geometry H (425), Adv Algebra II / Trig H (435), AP Precalculus (443), Adv Precalculus H (445), Calculus H (450), AP Calc AB (453), AP Calc BC (455), AP Statistics (456), Web Design (472), AP Computer Science A (490), AP Computer Science Principles (491), Applied Programming (494), AP Cybersecurity (496), Sports Medicine (544), AP Biology (551), AP Chemistry (553), AP Physics 1 (557), AP Physics C (558), Robotics Design (585), Robotics Project (590), Robotics Project II (591), Engineering Design (595), AP World History (713), Adv U.S. History I H (722), AP Business with Personal Finance (729), AP U.S. History (733), Leadership, Entrepreneurship and Opportunity Program I (734), AP European History (743), Sociology (744), Leadership, Entrepreneurship and Opportunity Program II (745), AP Psychology (761), AP U.S. Government &amp; Politics (763), AP Art History (764), AP Macroeconomics (765), AP Microeconomics (766), Academic Support (955)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Required Core / Graduation</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Required for graduation. Must be placed before lower priorities.</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Algebra I (410), Algebra I (412), American Literature (120), American Literature (122), British Literature (130), British Literature (132), Catholic Social Teaching (849), Composition &amp; Literature (110) ... (+10 more)</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Required Core / Grade-Level Mandate</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Required course mandated by grade level or graduation policy. Every student in the grade must complete it.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Composition &amp; Literature (110), Composition &amp; Literature (112), American Literature (120), American Literature (122), British Literature (130), British Literature (132), World Literature (140), Public Speaking (144), Journalism (145), World Literature (146), Algebra I (410), Algebra I (412), Geometry (420), Theology 9 (810), Theology 10 (820), Theology 11 (830), Catholic Social Teaching (849), Spirituality of Vocation (851)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Sequence / Honors / AP</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Academic sequence or advanced track. High placement priority.</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Algebra I H (411), Algebra II/Trig (430), Algebra II/Trig (432), Algebra II/Trig H (431), American Literature H (121), Anatomy/Physiology (542), Anatomy/Physiology H (543), Biology H (511) ... (+21 more)</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Sequence / Honors Track</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Progressive academic sequence or Honors-level track. Missing it delays academic progression by a year.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Composition &amp; Literature H (111), American Literature H (121), British Literature H (131), College English Honors (141), Multi-Media Production (2014), Italian I (312), Spanish II H (321), Italian II (322), Spanish III (330), Spanish III H (331), Italian III H (333), Algebra I H (411), Geometry H (421), Geometry (422), Algebra II/Trig (430), Algebra II/Trig H (431), Algebra II/Trig (432), Precalculus (440), Pre-college Math (448), Biology H (511), Chemistry H (521), Physics H (531), Anatomy/Physiology (542), Anatomy/Physiology H (543), World History H (711), U.S. History I H (721), U.S. History II H (731), Economics H (752), Introduction to Law (756)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Departmental Core</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Core departmental offerings. Important but not graduation-critical.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Biology (510), CPR-AED Training/PE (631), Chemistry (520), Driver's Ed/PE (620), Health/PE (610), Nutrition &amp; Fitness/PE (642), Physics (530), Psychology (741) ... (+5 more)</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Core departmental offering that fulfills graduation requirements. Multiple sections typically available.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Spanish I (310), Spanish II (320), Biology (510), Chemistry (520), Physics (530), Health/PE (610), Driver's Ed/PE (620), CPR-AED Training/PE (631), Nutrition &amp; Fitness/PE (642), World History (710), U.S. History I (720), U.S. History II (730), Psychology (741)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Standard Elective</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Elective courses. Placed after higher priorities satisfied.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>American Government &amp; Politics (751), Bloomberg Market Concepts (758), Business Concepts (726), Business Law (732), Digital Media (2054), Earth Science (500), Economics (742), Forensics (546) ... (+10 more)</t>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Elective — Standard</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Standard elective that enhances the program but is not required for graduation or sequence completion.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>TV/Film Process and Principles (2024), TV/Film Production &amp; Editing I (2034), TV/Film Production II (2044), Digital Media (2054), Studio Art I (241), Introduction to Programming (473), Earth Science (500), Forensics (546), Introduction to Robotics (570), Robotics Engineering (580), Introduction to Business (708), Business Concepts (726), Sports and Entertainment Marketing (727), Business Law (732), Economics (742), American Government &amp; Politics (751), International Business Strategies (757), Bloomberg Market Concepts (758)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Free Elective / Low Demand</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Nice-to-have. Placed last. Acceptable loss if conflicts exist.</t>
-        </is>
-      </c>
-      <c r="D10" s="3"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Elective — Flexible</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Non-essential elective with multiple scheduling alternatives. Can be dropped or rescheduled without academic impact.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -660,14 +652,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -677,11 +669,6 @@
           <t>8-INPUT WEIGHTED COMPOSITE SCORING SYSTEM</t>
         </is>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -689,316 +676,316 @@
           <t>Each student-course placement is scored using these 8 inputs</t>
         </is>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Course Flexibility Priority</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>CFP</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>How flexible is this course in scheduling?</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>How flexible is this course in scheduling? Single-section courses score higher.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Current Year Required Priority</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Current Year Request Priority</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>CYRP</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="5" t="n">
         <v>1.5</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Is this course required THIS year?</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Priority of the course request for the current academic year.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Student Special Priority</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Student Scheduling Priority</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>SSP</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Does this student have special scheduling needs?</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Individual student scheduling priority (IEP, senior status, etc.).</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Student Profile</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Master Teacher Priority</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MTP</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Is the assigned teacher highly constrained?</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-driven priority (department head, specialized instructor).</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Teacher Profile</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Course-Teacher Affinity Priority</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Course-Teacher Assignment Priority</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>CTAP</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="5" t="n">
         <v>1.5</v>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>How strong is the teacher-course match?</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Course + Teacher Profile</t>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Priority of assigning this specific teacher to this specific course.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Teacher Lock</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Teacher Load</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Is the teacher locked to specific periods?</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Teacher workload balancing factor. Higher = closer to overload.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Teacher Profile</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Period Lock</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Is this course locked to a specific period?</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>How constrained is the period assignment? 5 = must be specific period.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Course Profile</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Room Lock</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>RL</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="5" t="n">
         <v>1.5</v>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Is this course locked to a specific room?</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Room assignment constraint. Labs, gyms score higher.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Room Profile</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-    </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Maximum Weighted Sum:</t>
-        </is>
-      </c>
-      <c r="B14" s="5">
-        <f> 5x(1.0 + 1.5 + 2.0 + 1.0 + 1.5 + 2.0 + 2.0 + 1.5) = 62.5</f>
-        <v/>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>COMPOSITE FORMULA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>WS = CFP(x1.0) + CYRP(x1.5) + SSP(x2.0) + MTP(x1.0) + CTAP(x1.5) + TL(x2.0) + PL(x2.0) + RL(x1.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CC = count of inputs scoring &gt;= 4 (critical count). Max WS = 62.5, Max CC = 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Students ranked by: (1) max CC across all courses, (2) total WS across all courses. Bump decisions use (-CC, -WS) so highest-priority placements are protected.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>